<commit_message>
Fix: deadline dates were stored as strings, breaking date math reliability
</commit_message>
<xml_diff>
--- a/downloads/smlsheets/SMLSheets_GrantForge_Beastmode.xlsx
+++ b/downloads/smlsheets/SMLSheets_GrantForge_Beastmode.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="118">
   <si>
     <t xml:space="preserve">SMLSHEETS.AI — GRANT FORGE BEASTMODE</t>
   </si>
@@ -203,9 +203,6 @@
     <t xml:space="preserve">Federal SBIR</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-15</t>
-  </si>
-  <si>
     <t xml:space="preserve">High</t>
   </si>
   <si>
@@ -233,9 +230,6 @@
     <t xml:space="preserve">State Grant</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-08-01</t>
-  </si>
-  <si>
     <t xml:space="preserve">grants@ncidea.org</t>
   </si>
   <si>
@@ -254,9 +248,6 @@
     <t xml:space="preserve">Veteran Grant</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-07-20</t>
-  </si>
-  <si>
     <t xml:space="preserve">Yes</t>
   </si>
   <si>
@@ -275,9 +266,6 @@
     <t xml:space="preserve">FedEx</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-01</t>
-  </si>
-  <si>
     <t xml:space="preserve">Medium</t>
   </si>
   <si>
@@ -291,9 +279,6 @@
   </si>
   <si>
     <t xml:space="preserve">Federal Certification</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-12-31</t>
   </si>
   <si>
     <t xml:space="preserve">vetcert@sba.gov</t>
@@ -1388,8 +1373,8 @@
       <c r="C3" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="13" t="s">
-        <v>59</v>
+      <c r="D3" s="13" t="n">
+        <v>46280</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>300000</v>
@@ -1398,13 +1383,13 @@
         <v>32</v>
       </c>
       <c r="G3" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="H3" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="H3" s="12" t="s">
+      <c r="I3" s="12" t="s">
         <v>61</v>
-      </c>
-      <c r="I3" s="12" t="s">
-        <v>62</v>
       </c>
       <c r="J3" s="15" t="n">
         <f aca="true">D3-TODAY()</f>
@@ -1415,27 +1400,27 @@
         <v>4</v>
       </c>
       <c r="L3" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="M3" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="M3" s="12" t="s">
+      <c r="N3" s="13" t="s">
         <v>64</v>
-      </c>
-      <c r="N3" s="13" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B4" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="C4" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="C4" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>69</v>
+      <c r="D4" s="13" t="n">
+        <v>46235</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>50000</v>
@@ -1444,10 +1429,10 @@
         <v>31</v>
       </c>
       <c r="G4" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="H4" s="12" t="s">
         <v>60</v>
-      </c>
-      <c r="H4" s="12" t="s">
-        <v>61</v>
       </c>
       <c r="I4" s="12"/>
       <c r="J4" s="15" t="n">
@@ -1459,27 +1444,27 @@
         <v>4</v>
       </c>
       <c r="L4" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="M4" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="N4" s="13" t="s">
         <v>70</v>
-      </c>
-      <c r="M4" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="N4" s="13" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="B5" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>76</v>
+      <c r="D5" s="13" t="n">
+        <v>46223</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>25000</v>
@@ -1488,10 +1473,10 @@
         <v>31</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="I5" s="12"/>
       <c r="J5" s="15" t="n">
@@ -1503,27 +1488,27 @@
         <v>5</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="N5" s="13" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>83</v>
+        <v>73</v>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>46296</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>25000</v>
@@ -1532,10 +1517,10 @@
         <v>31</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I6" s="12"/>
       <c r="J6" s="15" t="n">
@@ -1548,24 +1533,24 @@
       </c>
       <c r="L6" s="12"/>
       <c r="M6" s="12" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="N6" s="13" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>89</v>
+        <v>84</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>46387</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>0</v>
@@ -1574,10 +1559,10 @@
         <v>31</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="I7" s="12"/>
       <c r="J7" s="15" t="n">
@@ -1589,13 +1574,13 @@
         <v>4</v>
       </c>
       <c r="L7" s="12" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="M7" s="12" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="N7" s="13" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2098,7 +2083,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -2106,13 +2091,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>41</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>54</v>
@@ -2120,76 +2105,76 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C6" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D6" s="12" t="s">
         <v>98</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="12" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="12" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="12"/>
@@ -2242,62 +2227,62 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B1" s="11"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>